<commit_message>
load spec files for antenna, add site name old and site name old
</commit_message>
<xml_diff>
--- a/backend/templates/template_cell_3g.xlsx
+++ b/backend/templates/template_cell_3g.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Cells_3G" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Cells_3G'!$A$1:$X$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Cells_3G'!$A$1:$Z$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X3"/>
+  <dimension ref="A1:Z3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -525,25 +525,27 @@
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="25" customWidth="1" min="4" max="4"/>
     <col width="25" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
     <col width="15" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="10" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
-    <col width="12" customWidth="1" min="16" max="16"/>
-    <col width="30" customWidth="1" min="17" max="17"/>
-    <col width="18" customWidth="1" min="18" max="18"/>
-    <col width="18" customWidth="1" min="19" max="19"/>
-    <col width="14" customWidth="1" min="20" max="20"/>
-    <col width="14" customWidth="1" min="21" max="21"/>
-    <col width="12" customWidth="1" min="22" max="22"/>
-    <col width="10" customWidth="1" min="23" max="23"/>
-    <col width="10" customWidth="1" min="24" max="24"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="15" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
+    <col width="10" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="30" customWidth="1" min="19" max="19"/>
+    <col width="18" customWidth="1" min="20" max="20"/>
+    <col width="18" customWidth="1" min="21" max="21"/>
+    <col width="14" customWidth="1" min="22" max="22"/>
+    <col width="14" customWidth="1" min="23" max="23"/>
+    <col width="12" customWidth="1" min="24" max="24"/>
+    <col width="10" customWidth="1" min="25" max="25"/>
+    <col width="10" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
@@ -562,107 +564,117 @@
           <t>Phuong xa</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Site Name Old</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Cell Name Old</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>Site Name</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>Cell Name</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Cell VIP</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>MORAN</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Lat</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Long</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Vung phu song</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Vendor</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Do cao anten</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Azimuth</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>M-tilt</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>E-Tilt</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Total Tilt</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Loai Anten</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Chung anten</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Baseband</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>RF</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Cell ID</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>ARFCN</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>PSC</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>MIMO</t>
         </is>
@@ -671,7 +683,7 @@
     <row r="2" ht="28" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Ghi chu: Cot mau VANG la bat buoc. Site Name phai ton tai hoac se duoc tu dong tao. Lat: 8.33-23.39, Long: 102.14-109.47. Azimuth: 0-359. Vendor: Ericsson/Nokia/Huawei/ZTE/Samsung. Vung phu song: Indoor/Outdoor. MIMO: 2x2/4x4/8x8.</t>
+          <t>Ghi chu: Cot mau VANG la bat buoc. Site Name phai ton tai hoac se duoc tu dong tao. Site Name Old / Cell Name Old: ten cu truoc khi doi (tuy chon). Lat: 8.33-23.39, Long: 102.14-109.47. Azimuth: 0-359. Vendor: Ericsson/Nokia/Huawei/ZTE/Samsung. Vung phu song: Indoor/Outdoor. MIMO: 2x2/4x4/8x8.</t>
         </is>
       </c>
       <c r="B2" s="4" t="n"/>
@@ -696,7 +708,9 @@
       <c r="U2" s="4" t="n"/>
       <c r="V2" s="4" t="n"/>
       <c r="W2" s="4" t="n"/>
-      <c r="X2" s="5" t="n"/>
+      <c r="X2" s="4" t="n"/>
+      <c r="Y2" s="4" t="n"/>
+      <c r="Z2" s="5" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -716,96 +730,106 @@
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
+          <t>HN-001-OLD</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>HN-001-3G-1-OLD</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
           <t>HN-001</t>
         </is>
       </c>
-      <c r="E3" s="6" t="inlineStr">
+      <c r="G3" s="6" t="inlineStr">
         <is>
           <t>HN-001-3G-1</t>
         </is>
       </c>
-      <c r="F3" s="6" t="inlineStr"/>
-      <c r="G3" s="6" t="inlineStr">
+      <c r="H3" s="6" t="inlineStr"/>
+      <c r="I3" s="6" t="inlineStr">
         <is>
           <t>MBF HOST</t>
         </is>
       </c>
-      <c r="H3" s="6" t="n">
+      <c r="J3" s="6" t="n">
         <v>21.0285</v>
       </c>
-      <c r="I3" s="6" t="n">
+      <c r="K3" s="6" t="n">
         <v>105.8542</v>
       </c>
-      <c r="J3" s="6" t="inlineStr">
+      <c r="L3" s="6" t="inlineStr">
         <is>
           <t>Outdoor</t>
         </is>
       </c>
-      <c r="K3" s="6" t="inlineStr">
+      <c r="M3" s="6" t="inlineStr">
         <is>
           <t>Huawei</t>
         </is>
       </c>
-      <c r="L3" s="6" t="n">
+      <c r="N3" s="6" t="n">
         <v>30</v>
       </c>
-      <c r="M3" s="6" t="n">
+      <c r="O3" s="6" t="n">
         <v>45</v>
-      </c>
-      <c r="N3" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="O3" s="6" t="n">
-        <v>0</v>
       </c>
       <c r="P3" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="Q3" s="6" t="inlineStr">
+      <c r="Q3" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R3" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="S3" s="6" t="inlineStr">
         <is>
           <t>Huawei ATR4518R10v06</t>
         </is>
       </c>
-      <c r="R3" s="6" t="inlineStr">
+      <c r="T3" s="6" t="inlineStr">
         <is>
           <t>3G</t>
         </is>
       </c>
-      <c r="S3" s="6" t="inlineStr">
+      <c r="U3" s="6" t="inlineStr">
         <is>
           <t>BBU3910</t>
         </is>
       </c>
-      <c r="T3" s="6" t="inlineStr">
+      <c r="V3" s="6" t="inlineStr">
         <is>
           <t>RRU3908</t>
         </is>
       </c>
-      <c r="U3" s="6" t="inlineStr">
+      <c r="W3" s="6" t="inlineStr">
         <is>
           <t>12345</t>
         </is>
       </c>
-      <c r="V3" s="6" t="inlineStr">
+      <c r="X3" s="6" t="inlineStr">
         <is>
           <t>10562</t>
         </is>
       </c>
-      <c r="W3" s="6" t="inlineStr">
+      <c r="Y3" s="6" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
-      <c r="X3" s="6" t="inlineStr">
+      <c r="Z3" s="6" t="inlineStr">
         <is>
           <t>2x2</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:X1"/>
+  <autoFilter ref="A1:Z1"/>
   <mergeCells count="1">
-    <mergeCell ref="A2:X2"/>
+    <mergeCell ref="A2:Z2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
change excel template to add drop list and data validation
</commit_message>
<xml_diff>
--- a/backend/templates/template_cell_3g.xlsx
+++ b/backend/templates/template_cell_3g.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -37,13 +37,8 @@
       <color rgb="007B3F00"/>
       <sz val="11"/>
     </font>
-    <font>
-      <i val="1"/>
-      <color rgb="00375623"/>
-      <sz val="10"/>
-    </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -60,13 +55,8 @@
         <fgColor rgb="00FFE699"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="6">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -88,55 +78,11 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="00BFBFBF"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00BFBFBF"/>
-      </right>
-      <top style="thin">
-        <color rgb="00BFBFBF"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="00BFBFBF"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00BFBFBF"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00BFBFBF"/>
-      </right>
-      <top style="thin">
-        <color rgb="00BFBFBF"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00BFBFBF"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -144,11 +90,6 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -517,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z3"/>
+  <dimension ref="A1:Z2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -680,147 +621,115 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="28" customHeight="1">
+    <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Ghi chu: Cot mau VANG la bat buoc. Site Name phai ton tai hoac se duoc tu dong tao. Site Name Old / Cell Name Old: ten cu truoc khi doi (tuy chon). Lat: 8.33-23.39, Long: 102.14-109.47. Azimuth: 0-359. Vendor: Ericsson/Nokia/Huawei/ZTE/Samsung. Vung phu song: Indoor/Outdoor. MIMO: 2x2/4x4/8x8.</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="n"/>
-      <c r="C2" s="4" t="n"/>
-      <c r="D2" s="4" t="n"/>
-      <c r="E2" s="4" t="n"/>
-      <c r="F2" s="4" t="n"/>
-      <c r="G2" s="4" t="n"/>
-      <c r="H2" s="4" t="n"/>
-      <c r="I2" s="4" t="n"/>
-      <c r="J2" s="4" t="n"/>
-      <c r="K2" s="4" t="n"/>
-      <c r="L2" s="4" t="n"/>
-      <c r="M2" s="4" t="n"/>
-      <c r="N2" s="4" t="n"/>
-      <c r="O2" s="4" t="n"/>
-      <c r="P2" s="4" t="n"/>
-      <c r="Q2" s="4" t="n"/>
-      <c r="R2" s="4" t="n"/>
-      <c r="S2" s="4" t="n"/>
-      <c r="T2" s="4" t="n"/>
-      <c r="U2" s="4" t="n"/>
-      <c r="V2" s="4" t="n"/>
-      <c r="W2" s="4" t="n"/>
-      <c r="X2" s="4" t="n"/>
-      <c r="Y2" s="4" t="n"/>
-      <c r="Z2" s="5" t="n"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
           <t>MB</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>Ha Noi</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>Phuong Trung Hoa</t>
         </is>
       </c>
-      <c r="D3" s="6" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>HN-001-OLD</t>
         </is>
       </c>
-      <c r="E3" s="6" t="inlineStr">
+      <c r="E2" s="3" t="inlineStr">
         <is>
           <t>HN-001-3G-1-OLD</t>
         </is>
       </c>
-      <c r="F3" s="6" t="inlineStr">
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>HN-001</t>
         </is>
       </c>
-      <c r="G3" s="6" t="inlineStr">
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>HN-001-3G-1</t>
         </is>
       </c>
-      <c r="H3" s="6" t="inlineStr"/>
-      <c r="I3" s="6" t="inlineStr">
+      <c r="H2" s="3" t="inlineStr"/>
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>MBF HOST</t>
         </is>
       </c>
-      <c r="J3" s="6" t="n">
+      <c r="J2" s="3" t="n">
         <v>21.0285</v>
       </c>
-      <c r="K3" s="6" t="n">
+      <c r="K2" s="3" t="n">
         <v>105.8542</v>
       </c>
-      <c r="L3" s="6" t="inlineStr">
+      <c r="L2" s="3" t="inlineStr">
         <is>
           <t>Outdoor</t>
         </is>
       </c>
-      <c r="M3" s="6" t="inlineStr">
+      <c r="M2" s="3" t="inlineStr">
         <is>
           <t>Huawei</t>
         </is>
       </c>
-      <c r="N3" s="6" t="n">
+      <c r="N2" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="O3" s="6" t="n">
+      <c r="O2" s="3" t="n">
         <v>45</v>
       </c>
-      <c r="P3" s="6" t="n">
+      <c r="P2" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="Q3" s="6" t="n">
+      <c r="Q2" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="R3" s="6" t="n">
+      <c r="R2" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="S3" s="6" t="inlineStr">
+      <c r="S2" s="3" t="inlineStr">
         <is>
           <t>Huawei ATR4518R10v06</t>
         </is>
       </c>
-      <c r="T3" s="6" t="inlineStr">
+      <c r="T2" s="3" t="inlineStr">
         <is>
           <t>3G</t>
         </is>
       </c>
-      <c r="U3" s="6" t="inlineStr">
+      <c r="U2" s="3" t="inlineStr">
         <is>
           <t>BBU3910</t>
         </is>
       </c>
-      <c r="V3" s="6" t="inlineStr">
+      <c r="V2" s="3" t="inlineStr">
         <is>
           <t>RRU3908</t>
         </is>
       </c>
-      <c r="W3" s="6" t="inlineStr">
+      <c r="W2" s="3" t="inlineStr">
         <is>
           <t>12345</t>
         </is>
       </c>
-      <c r="X3" s="6" t="inlineStr">
+      <c r="X2" s="3" t="inlineStr">
         <is>
           <t>10562</t>
         </is>
       </c>
-      <c r="Y3" s="6" t="inlineStr">
+      <c r="Y2" s="3" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
-      <c r="Z3" s="6" t="inlineStr">
+      <c r="Z2" s="3" t="inlineStr">
         <is>
           <t>2x2</t>
         </is>
@@ -828,9 +737,41 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:Z1"/>
-  <mergeCells count="1">
-    <mergeCell ref="A2:Z2"/>
-  </mergeCells>
+  <dataValidations count="10">
+    <dataValidation sqref="A2:A1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Giá trị không hợp lệ" error="Vui lòng chọn từ danh sách" type="list">
+      <formula1>"MB,MT,MN"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H2:H1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Giá trị không hợp lệ" error="Vui lòng chọn từ danh sách" type="list">
+      <formula1>"VIP,VVIP"</formula1>
+    </dataValidation>
+    <dataValidation sqref="I2:I1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Giá trị không hợp lệ" error="Chọn: VNPT HOST hoặc MBF HOST" type="list">
+      <formula1>"VNPT HOST,MBF HOST"</formula1>
+    </dataValidation>
+    <dataValidation sqref="J2:J1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Giá trị ngoài phạm vi" error="Latitude phải trong khoảng 8.33–23.39" type="decimal" errorStyle="warning" operator="between">
+      <formula1>8.33</formula1>
+      <formula2>23.39</formula2>
+    </dataValidation>
+    <dataValidation sqref="K2:K1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Giá trị ngoài phạm vi" error="Longitude phải trong khoảng 102.14–109.47" type="decimal" errorStyle="warning" operator="between">
+      <formula1>102.14</formula1>
+      <formula2>109.47</formula2>
+    </dataValidation>
+    <dataValidation sqref="L2:L1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Giá trị không hợp lệ" error="Vui lòng chọn từ danh sách" type="list">
+      <formula1>"Indoor,Outdoor"</formula1>
+    </dataValidation>
+    <dataValidation sqref="M2:M1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Giá trị không hợp lệ" error="Vui lòng chọn từ danh sách" type="list">
+      <formula1>"Ericsson,Nokia,Huawei,ZTE,Samsung"</formula1>
+    </dataValidation>
+    <dataValidation sqref="O2:O1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Giá trị ngoài phạm vi" error="Azimuth phải trong khoảng 0–359" type="whole" errorStyle="warning" operator="between">
+      <formula1>0</formula1>
+      <formula2>359</formula2>
+    </dataValidation>
+    <dataValidation sqref="T2:T1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Giá trị không hợp lệ" error="Chọn: 3G, 3G/4G, 2G/3G/4G, 3G/4G/5G, 3G/5G" type="list">
+      <formula1>"3G,3G/4G,2G/3G/4G,3G/4G/5G,3G/5G"</formula1>
+    </dataValidation>
+    <dataValidation sqref="Z2:Z1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Giá trị không hợp lệ" error="Vui lòng chọn từ danh sách" type="list">
+      <formula1>"2x2,4x4,8x8"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
add columns for cells
</commit_message>
<xml_diff>
--- a/backend/templates/template_cell_3g.xlsx
+++ b/backend/templates/template_cell_3g.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Cells_3G" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Cells_3G'!$A$1:$Z$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Cells_3G'!$A$1:$AG$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z2"/>
+  <dimension ref="A1:AG2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -487,6 +487,13 @@
     <col width="12" customWidth="1" min="24" max="24"/>
     <col width="10" customWidth="1" min="25" max="25"/>
     <col width="10" customWidth="1" min="26" max="26"/>
+    <col width="10" customWidth="1" min="27" max="27"/>
+    <col width="10" customWidth="1" min="28" max="28"/>
+    <col width="10" customWidth="1" min="29" max="29"/>
+    <col width="20" customWidth="1" min="30" max="30"/>
+    <col width="18" customWidth="1" min="31" max="31"/>
+    <col width="16" customWidth="1" min="32" max="32"/>
+    <col width="24" customWidth="1" min="33" max="33"/>
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
@@ -607,17 +614,52 @@
       </c>
       <c r="X1" s="1" t="inlineStr">
         <is>
-          <t>ARFCN</t>
+          <t>UARFCN</t>
         </is>
       </c>
       <c r="Y1" s="1" t="inlineStr">
         <is>
+          <t>LAC</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>RAC</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
           <t>PSC</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>MIMO</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>URAId</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>Cell max power (dBm)</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>CPICH power (dBm)</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>BBUname</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>Cell status (at dump time)</t>
         </is>
       </c>
     </row>
@@ -726,17 +768,52 @@
       </c>
       <c r="Y2" s="3" t="inlineStr">
         <is>
+          <t>1234</t>
+        </is>
+      </c>
+      <c r="Z2" s="3" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="AA2" s="3" t="inlineStr">
+        <is>
           <t>100</t>
         </is>
       </c>
-      <c r="Z2" s="3" t="inlineStr">
+      <c r="AB2" s="3" t="inlineStr">
         <is>
           <t>2x2</t>
+        </is>
+      </c>
+      <c r="AC2" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AD2" s="3" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="AE2" s="3" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="AF2" s="3" t="inlineStr">
+        <is>
+          <t>BBU-HN-001</t>
+        </is>
+      </c>
+      <c r="AG2" s="3" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Z1"/>
+  <autoFilter ref="A1:AG1"/>
   <dataValidations count="10">
     <dataValidation sqref="A2:A1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Giá trị không hợp lệ" error="Vui lòng chọn từ danh sách" type="list">
       <formula1>"MB,MT,MN"</formula1>
@@ -744,14 +821,14 @@
     <dataValidation sqref="H2:H1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Giá trị không hợp lệ" error="Vui lòng chọn từ danh sách" type="list">
       <formula1>"VIP,VVIP"</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Giá trị không hợp lệ" error="Chọn: VNPT HOST hoặc MBF HOST" type="list">
+    <dataValidation sqref="I2:I1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Giá trị không hợp lệ" error="Vui lòng chọn từ danh sách" type="list">
       <formula1>"VNPT HOST,MBF HOST"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Giá trị ngoài phạm vi" error="Latitude phải trong khoảng 8.33–23.39" type="decimal" errorStyle="warning" operator="between">
+    <dataValidation sqref="J2:J1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Giá trị ngoài phạm vi" error="Giá trị ngoài phạm vi" type="decimal" errorStyle="warning" operator="between">
       <formula1>8.33</formula1>
       <formula2>23.39</formula2>
     </dataValidation>
-    <dataValidation sqref="K2:K1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Giá trị ngoài phạm vi" error="Longitude phải trong khoảng 102.14–109.47" type="decimal" errorStyle="warning" operator="between">
+    <dataValidation sqref="K2:K1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Giá trị ngoài phạm vi" error="Giá trị ngoài phạm vi" type="decimal" errorStyle="warning" operator="between">
       <formula1>102.14</formula1>
       <formula2>109.47</formula2>
     </dataValidation>
@@ -761,14 +838,14 @@
     <dataValidation sqref="M2:M1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Giá trị không hợp lệ" error="Vui lòng chọn từ danh sách" type="list">
       <formula1>"Ericsson,Nokia,Huawei,ZTE,Samsung"</formula1>
     </dataValidation>
-    <dataValidation sqref="O2:O1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Giá trị ngoài phạm vi" error="Azimuth phải trong khoảng 0–359" type="whole" errorStyle="warning" operator="between">
+    <dataValidation sqref="O2:O1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Giá trị ngoài phạm vi" error="Giá trị ngoài phạm vi" type="whole" errorStyle="warning" operator="between">
       <formula1>0</formula1>
       <formula2>359</formula2>
     </dataValidation>
-    <dataValidation sqref="T2:T1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Giá trị không hợp lệ" error="Chọn: 3G, 3G/4G, 2G/3G/4G, 3G/4G/5G, 3G/5G" type="list">
+    <dataValidation sqref="T2:T1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Giá trị không hợp lệ" error="Vui lòng chọn từ danh sách" type="list">
       <formula1>"3G,3G/4G,2G/3G/4G,3G/4G/5G,3G/5G"</formula1>
     </dataValidation>
-    <dataValidation sqref="Z2:Z1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Giá trị không hợp lệ" error="Vui lòng chọn từ danh sách" type="list">
+    <dataValidation sqref="AB2:AB1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Giá trị không hợp lệ" error="Vui lòng chọn từ danh sách" type="list">
       <formula1>"2x2,4x4,8x8"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>